<commit_message>
NOVA GRAVITY v1.01: portfolio sharing, weekly limit, adaptive risk, rollover guard, journal CSV, OnTester + Monte Carlo analytics
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/NovaGravity_AI/Excel/NovaGravity_AI_Settings.xlsx
+++ b/NovaGravity_AI/Excel/NovaGravity_AI_Settings.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="01 - Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="02 - Full Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02 - Full Inputs1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03 - Risk &amp; MM" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04 - Symbol Classes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05 - Friday Weekend" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06 - Presets" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07 - Runbook" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="03 - Risk &amp; MM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04 - Symbol Classes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05 - Friday Weekend" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="06 - Presets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="07 - Runbook" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="08 - Portfolio &amp; Journal" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="08 - Changelog" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
@@ -494,7 +494,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.00 (Pro)</t>
+          <t>1.01 (Pro + Portfolio)</t>
         </is>
       </c>
     </row>
@@ -665,20 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3277,12 +3264,372 @@
       </c>
       <c r="G86" s="5" t="inlineStr"/>
     </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>InpPortfolioSharing</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Share day/week limits across ALL charts of the EA</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>InpWeeklyLossLimitPercent</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Weekly loss limit % (0=off) - portfolio-wide</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveRisk</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Auto-reduce risk as drawdown grows</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>InpRiskReductionStartDD</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Drawdown % where risk scaling starts</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>InpRiskReductionFloor</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Minimum risk multiplier (never below this)</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>InpRolloverGuard</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Guard against negative swap at rollover</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>InpRolloverStart</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Rollover start (server hour)</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>InpRolloverEnd</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Rollover end (server hour)</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>InpRolloverSwapThreshold</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Trigger if position swap &lt; this ($)</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>InpRolloverAction</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>ENUM_NG_ROLLOVER_ACTION</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>NG_ROLLOVER_BREAKEVEN</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Guard action</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>InpJournalCSV</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Write NovaGravity_Journal.csv (MQL5/Files)</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="4">
+        <f>==== 09 | PORTFOLIO SHARING &amp; JOURNAL =====</f>
+        <v/>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>InpNotifyOnGuards</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Push notification on critical events</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3437,7 +3784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3747,7 +4094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3885,13 +4232,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3967,12 +4314,80 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>IC Markets</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>NovaGravity_AI_IC_Markets.set</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Tight spreads: filter 0.10 ATR, deviation 10, GMT+3, sessions ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pepperstone</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>NovaGravity_AI_Pepperstone.set</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Spread filter 0.12 ATR, deviation 15, GMT+3, sessions ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Exness</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>NovaGravity_AI_Exness.set</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Spread filter 0.18 ATR, risk 0.7%, auto GMT offset, sessions ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>PROP CHALLENGE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>NovaGravity_AI_Prop_Challenge.set</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Risk 0.5%, daily 4%, weekly 8%, global DD stop 10%, adaptive risk from 3% DD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4110,13 +4525,253 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>InpPortfolioSharing</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Shares day/week P/L across ALL charts running the EA via terminal global variables (cross-chart protection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>InpWeeklyLossLimitPercent</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Portfolio weekly loss limit - closes all + halts until Monday (0=off)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>InpAdaptiveRisk</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Risk scales DOWN as equity drawdown grows (never martingale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>InpRiskReductionStartDD</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Drawdown % where risk reduction begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>InpRiskReductionFloor</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Minimum risk multiplier (25% of configured risk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>InpRolloverGuard</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Rollover window protection for negative-swap positions (gold/oil) - BE or close</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>InpRolloverStart/End</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>21 / 22</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Rollover window in server hours (wrap-safe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>InpRolloverSwapThreshold</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Trigger when accumulated position swap &lt; -0.5 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>InpRolloverAction</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>BREAKEVEN</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Action: BE (default) or CLOSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>InpJournalCSV</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Writes MQL5/Files/NovaGravity_Journal.csv (imports into the dashboard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>InpNotifyOnGuards</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SendNotification push alerts on guard activations (needs MetaQuotes ID)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>OnTester()</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>built-in</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Custom optimizer criterion = PF x sqrt(N) / maxDD% - select Custom criterion in the tester</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4144,15 +4799,32 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
+          <t>v1.01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Portfolio sharing (cross-chart day/week limits via terminal globals), weekly loss limit, adaptive risk scaling with drawdown, rollover/swap guard, EA trade journal CSV (MQL5/Files), OnTester custom criterion PF x sqrt(N)/DD, weekly server-offset re-detect (DST), push notifications, broker/prop preset profiles (IC/Pepperstone/Exness/Prop Challenge). Dashboard: Monte Carlo bootstrap, overfitting check, Sortino/Kelly/max-consecutive-losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
           <t>v1.00</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Complete rebuild: auto symbol-class &amp; timeframe detection; Friday weekend guard (close/BE 1h before cutoff); QUIET=wait &amp; VOLATILE=range-only; partial -&gt; immediate breakeven lock; per-class max-hold time stop; gap filter extended to gold/oil/all classes; news blackout (13-16 server, extended Friday, crypto exempt); server GMT offset auto-detect; VOLUME_STEP lot rounding; pullback EMA21/55 + BB mid entries with HTF alignment; anti-chase filter; daily loss limit; optional global DD stop; on-chart panel.</t>
         </is>

</xml_diff>

<commit_message>
NOVA GRAVITY v1.02: profit ladder, 4 trail modes, equity guard, adaptive AI engine, sounds, new logo + chart dashboard
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/NovaGravity_AI/Excel/NovaGravity_AI_Settings.xlsx
+++ b/NovaGravity_AI/Excel/NovaGravity_AI_Settings.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.01 (Pro + Portfolio)</t>
+          <t>1.02 (Pro + Engines + AI)</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3623,6 +3623,756 @@
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>InpProfitLadderEnabled</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>4-degree profit ladder (auto-adaptive)</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung1Points</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Rung 1: profit points</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung1Percent</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Rung 1: % of volume closed</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung2Points</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Rung 2: profit points</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung2Percent</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Rung 2: % of remaining closed</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung3Points</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Rung 3: profit points</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung3Percent</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Rung 3: % of remaining closed</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung4Points</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Rung 4: profit points</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>InpLadderRung4Percent</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Rung 4: % of remaining closed</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>InpTrailMode</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>ENUM_NG_TRAIL_MODE</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>NG_TRAIL_ATR</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Trailing mode (ATR | POINTS | PERCENT | LADDER)</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>InpTrailFixedPoints</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>TRAIL_POINTS: move SL after +X points</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>InpTrailPercentStep</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>TRAIL_PERCENT: move SL at +% of profit-to-TP</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>InpEquityGuardEnabled</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Equity Guard card (modeled on the reference panel)</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>InpGuardDailyLossPct</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>Equity Guard: daily loss % goal</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>InpGuardMaxDrawdownPct</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Equity Guard: max drawdown % goal</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>InpGuardMinFreeMarginPct</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Equity Guard: minimum free-margin % floor</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="4">
+        <f>==== 10 | PROFIT ENGINES: LADDER / TRAIL / EQUITY GUARD =====</f>
+        <v/>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>InpGuardMinHedgePct</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Equity Guard: minimum hedged % (info card)</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveEngine</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Self-learning optimizer (auto-tunes &amp; filters positive results)</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveEvalEvery</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Evaluate candidate genomes every N closed trades</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveMinSamples</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Min closed trades before a candidate is trusted</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveImprovePct</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Switch only if new score beats current by %</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptivePersist</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>Save best genome + history to MQL5/Files</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>InpAdaptiveReset</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Reset learned state on init</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>InpSoundAlerts</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Audible alerts (PlaySound)</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="4">
+        <f>==== 11 | ADAPTIVE AI ENGINE (self-learning optimization) =====</f>
+        <v/>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>InpCustomSound</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>"NovaGravity_alert.wav"</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Custom sound (MQL5/Sounds); falls back to alert.wav</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>